<commit_message>
attempting longer training to increase accuracy
</commit_message>
<xml_diff>
--- a/documentation/Training statistics.xlsx
+++ b/documentation/Training statistics.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="33">
   <si>
     <t>Training experiments - Chokepoint camera</t>
   </si>
@@ -84,6 +84,45 @@
   </si>
   <si>
     <t>Best</t>
+  </si>
+  <si>
+    <t>Training time</t>
+  </si>
+  <si>
+    <t>3 hrs</t>
+  </si>
+  <si>
+    <t>1 hr</t>
+  </si>
+  <si>
+    <t>40 mins</t>
+  </si>
+  <si>
+    <t>4.5 hrs</t>
+  </si>
+  <si>
+    <t>1.5 hrs</t>
+  </si>
+  <si>
+    <t>~2 hrs</t>
+  </si>
+  <si>
+    <t>6 hrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">13 hrs </t>
+  </si>
+  <si>
+    <t>Epochs</t>
+  </si>
+  <si>
+    <t>50 + 20</t>
+  </si>
+  <si>
+    <t>200 + 40</t>
+  </si>
+  <si>
+    <t>Automatic</t>
   </si>
 </sst>
 </file>
@@ -213,19 +252,13 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -242,6 +275,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -524,77 +563,87 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:M27"/>
+  <dimension ref="B2:O27"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.08984375" customWidth="1"/>
-    <col min="3" max="3" width="17.7265625" customWidth="1"/>
-    <col min="4" max="7" width="14.54296875" customWidth="1"/>
-    <col min="8" max="8" width="14.1796875" customWidth="1"/>
-    <col min="9" max="9" width="14.6328125" customWidth="1"/>
+    <col min="3" max="5" width="17.7265625" customWidth="1"/>
+    <col min="6" max="9" width="14.54296875" customWidth="1"/>
+    <col min="10" max="10" width="14.1796875" customWidth="1"/>
+    <col min="11" max="11" width="14.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B2" s="8" t="s">
+    <row r="2" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B2" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-    </row>
-    <row r="4" spans="2:13" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="4" t="s">
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
+      <c r="J2" s="4"/>
+      <c r="K2" s="4"/>
+      <c r="L2" s="4"/>
+      <c r="M2" s="4"/>
+    </row>
+    <row r="4" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="9" t="s">
+      <c r="G4" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F4" s="10"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="12" t="s">
+      <c r="H4" s="8"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="4" t="s">
+      <c r="K4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="J4" s="4" t="s">
+      <c r="L4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K4" s="6" t="s">
+      <c r="M4" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="2" t="s">
+    <row r="5" spans="2:15" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="13"/>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="2:13" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="J5" s="11"/>
+      <c r="K5" s="6"/>
+      <c r="L5" s="6"/>
+      <c r="M5" s="13"/>
+    </row>
+    <row r="6" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
         <v>46052</v>
       </c>
@@ -602,31 +651,37 @@
         <v>18</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="1">
+      <c r="G6" s="1">
         <v>33</v>
       </c>
-      <c r="F6" s="1">
+      <c r="H6" s="1">
         <v>12</v>
       </c>
-      <c r="G6" s="1">
+      <c r="I6" s="1">
         <v>5</v>
       </c>
-      <c r="H6" s="1">
+      <c r="J6" s="1">
         <v>116</v>
       </c>
-      <c r="I6" s="1">
+      <c r="K6" s="1">
         <v>0.21299999999999999</v>
       </c>
-      <c r="J6" s="1">
+      <c r="L6" s="1">
         <v>0.3</v>
       </c>
-      <c r="K6" s="1">
+      <c r="M6" s="1">
         <v>0.12</v>
       </c>
     </row>
-    <row r="7" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="7" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B7" s="3">
         <v>46052</v>
       </c>
@@ -634,34 +689,40 @@
         <v>11</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E7" s="1">
+      <c r="G7" s="1">
         <v>33</v>
       </c>
-      <c r="F7" s="1">
+      <c r="H7" s="1">
         <v>12</v>
       </c>
-      <c r="G7" s="1">
+      <c r="I7" s="1">
         <v>5</v>
       </c>
-      <c r="H7" s="1">
+      <c r="J7" s="1">
         <v>116</v>
       </c>
-      <c r="I7" s="1">
+      <c r="K7" s="1">
         <v>0.377</v>
       </c>
-      <c r="J7" s="1">
+      <c r="L7" s="1">
         <v>0.875</v>
       </c>
-      <c r="K7" s="1">
+      <c r="M7" s="1">
         <v>0.50900000000000001</v>
       </c>
-      <c r="M7" t="s">
+      <c r="O7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="8" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="8" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B8" s="3">
         <v>46057</v>
       </c>
@@ -669,34 +730,40 @@
         <v>18</v>
       </c>
       <c r="D8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="1">
+      <c r="G8" s="1">
         <v>128</v>
       </c>
-      <c r="F8" s="1">
+      <c r="H8" s="1">
         <v>44</v>
       </c>
-      <c r="G8" s="1">
+      <c r="I8" s="1">
         <v>20</v>
       </c>
-      <c r="H8" s="1">
+      <c r="J8" s="1">
         <v>448</v>
       </c>
-      <c r="I8" s="1">
+      <c r="K8" s="1">
         <v>0.40699999999999997</v>
       </c>
-      <c r="J8" s="1">
+      <c r="L8" s="1">
         <v>0.60799999999999998</v>
       </c>
-      <c r="K8" s="1">
+      <c r="M8" s="1">
         <v>0.42699999999999999</v>
       </c>
-      <c r="M8" t="s">
+      <c r="O8" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B9" s="3">
         <v>46059</v>
       </c>
@@ -704,31 +771,37 @@
         <v>11</v>
       </c>
       <c r="D9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E9" s="1">
+      <c r="G9" s="1">
         <v>128</v>
       </c>
-      <c r="F9" s="1">
+      <c r="H9" s="1">
         <v>44</v>
       </c>
-      <c r="G9" s="1">
+      <c r="I9" s="1">
         <v>20</v>
       </c>
-      <c r="H9" s="1">
+      <c r="J9" s="1">
         <v>448</v>
       </c>
-      <c r="I9" s="1">
+      <c r="K9" s="1">
         <v>0.495</v>
       </c>
-      <c r="J9" s="1">
+      <c r="L9" s="1">
         <v>0.497</v>
       </c>
-      <c r="K9" s="1">
+      <c r="M9" s="1">
         <v>0.41399999999999998</v>
       </c>
     </row>
-    <row r="10" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B10" s="3">
         <v>46071</v>
       </c>
@@ -736,31 +809,37 @@
         <v>11</v>
       </c>
       <c r="D10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E10" s="1">
+      <c r="G10" s="1">
         <v>236</v>
       </c>
-      <c r="F10" s="1">
+      <c r="H10" s="1">
         <v>114</v>
       </c>
-      <c r="G10" s="1">
+      <c r="I10" s="1">
         <v>49</v>
       </c>
-      <c r="H10" s="1">
+      <c r="J10" s="1">
         <v>871</v>
       </c>
-      <c r="I10" s="1">
+      <c r="K10" s="1">
         <v>0.49</v>
       </c>
-      <c r="J10" s="1">
+      <c r="L10" s="1">
         <v>0.50800000000000001</v>
       </c>
-      <c r="K10" s="1">
+      <c r="M10" s="1">
         <v>0.5</v>
       </c>
     </row>
-    <row r="11" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:15" x14ac:dyDescent="0.35">
       <c r="B11" s="3">
         <v>46071</v>
       </c>
@@ -768,46 +847,78 @@
         <v>18</v>
       </c>
       <c r="D11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F11" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="1">
+      <c r="G11" s="1">
         <v>236</v>
       </c>
-      <c r="F11" s="1">
+      <c r="H11" s="1">
         <v>114</v>
       </c>
-      <c r="G11" s="1">
+      <c r="I11" s="1">
         <v>49</v>
       </c>
-      <c r="H11" s="1">
+      <c r="J11" s="1">
         <v>871</v>
       </c>
-      <c r="I11" s="1">
+      <c r="K11" s="1">
         <v>0.44800000000000001</v>
       </c>
-      <c r="J11" s="1">
+      <c r="L11" s="1">
         <v>0.59799999999999998</v>
       </c>
-      <c r="K11" s="1">
+      <c r="M11" s="1">
         <v>0.46400000000000002</v>
       </c>
-      <c r="L11" t="s">
+      <c r="N11" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
-      <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-      <c r="K12" s="1"/>
-    </row>
-    <row r="13" spans="2:13" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B12" s="3">
+        <v>46077</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="1">
+        <v>236</v>
+      </c>
+      <c r="H12" s="1">
+        <v>114</v>
+      </c>
+      <c r="I12" s="1">
+        <v>49</v>
+      </c>
+      <c r="J12" s="1">
+        <v>871</v>
+      </c>
+      <c r="K12" s="1">
+        <v>0.47</v>
+      </c>
+      <c r="L12" s="1">
+        <v>0.55200000000000005</v>
+      </c>
+      <c r="M12" s="1">
+        <v>0.442</v>
+      </c>
+    </row>
+    <row r="13" spans="2:15" ht="13" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
@@ -818,68 +929,80 @@
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
-    </row>
-    <row r="16" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B16" s="8" t="s">
+      <c r="L13" s="1"/>
+      <c r="M13" s="1"/>
+    </row>
+    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B16" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
-      <c r="J16" s="8"/>
-      <c r="K16" s="8"/>
-    </row>
-    <row r="18" spans="2:12" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="4" t="s">
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
+      <c r="I16" s="4"/>
+      <c r="J16" s="4"/>
+      <c r="K16" s="4"/>
+      <c r="L16" s="4"/>
+      <c r="M16" s="4"/>
+    </row>
+    <row r="18" spans="2:14" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B18" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="4" t="s">
+      <c r="C18" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D18" s="4" t="s">
+      <c r="D18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E18" s="9" t="s">
+      <c r="G18" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="F18" s="10"/>
-      <c r="G18" s="11"/>
-      <c r="H18" s="12" t="s">
+      <c r="H18" s="8"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="I18" s="4" t="s">
+      <c r="K18" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="J18" s="4" t="s">
+      <c r="L18" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="K18" s="6" t="s">
+      <c r="M18" s="12" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="2:12" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="5"/>
-      <c r="C19" s="5"/>
-      <c r="D19" s="5"/>
-      <c r="E19" s="2" t="s">
+    <row r="19" spans="2:14" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="F19" s="2" t="s">
+      <c r="H19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="G19" s="2" t="s">
+      <c r="I19" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="H19" s="13"/>
-      <c r="I19" s="5"/>
-      <c r="J19" s="5"/>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="J19" s="11"/>
+      <c r="K19" s="6"/>
+      <c r="L19" s="6"/>
+      <c r="M19" s="13"/>
+    </row>
+    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B20" s="3">
         <v>46071</v>
       </c>
@@ -887,31 +1010,37 @@
         <v>11</v>
       </c>
       <c r="D20" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F20" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E20" s="1">
+      <c r="G20" s="1">
         <v>88</v>
       </c>
-      <c r="F20" s="1">
+      <c r="H20" s="1">
         <v>25</v>
       </c>
-      <c r="G20" s="1">
+      <c r="I20" s="1">
         <v>12</v>
       </c>
-      <c r="H20" s="1">
+      <c r="J20" s="1">
         <v>301</v>
       </c>
-      <c r="I20" s="1">
+      <c r="K20" s="1">
         <v>0.93200000000000005</v>
       </c>
-      <c r="J20" s="1">
+      <c r="L20" s="1">
         <v>0.72499999999999998</v>
       </c>
-      <c r="K20" s="1">
+      <c r="M20" s="1">
         <v>0.82599999999999996</v>
       </c>
     </row>
-    <row r="21" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="3">
         <v>46072</v>
       </c>
@@ -919,34 +1048,40 @@
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F21" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="E21" s="1">
+      <c r="G21" s="1">
         <v>189</v>
       </c>
-      <c r="F21" s="1">
+      <c r="H21" s="1">
         <v>72</v>
       </c>
-      <c r="G21" s="1">
+      <c r="I21" s="1">
         <v>31</v>
       </c>
-      <c r="H21" s="1">
+      <c r="J21" s="1">
         <v>704</v>
       </c>
-      <c r="I21" s="1">
+      <c r="K21" s="1">
         <v>0.94099999999999995</v>
       </c>
-      <c r="J21" s="1">
+      <c r="L21" s="1">
         <v>0.79600000000000004</v>
       </c>
-      <c r="K21" s="1">
+      <c r="M21" s="1">
         <v>0.88700000000000001</v>
       </c>
-      <c r="L21" t="s">
+      <c r="N21" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="2:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B22" s="3"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
@@ -957,8 +1092,10 @@
       <c r="I22" s="1"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
-    </row>
-    <row r="23" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+    </row>
+    <row r="23" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
@@ -969,8 +1106,10 @@
       <c r="I23" s="1"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
-    </row>
-    <row r="24" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+    </row>
+    <row r="24" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B24" s="3"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
@@ -981,8 +1120,10 @@
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
-    </row>
-    <row r="25" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+    </row>
+    <row r="25" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
@@ -993,8 +1134,10 @@
       <c r="I25" s="1"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
-    </row>
-    <row r="26" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+    </row>
+    <row r="26" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
@@ -1005,8 +1148,10 @@
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
-    </row>
-    <row r="27" spans="2:12" x14ac:dyDescent="0.35">
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+    </row>
+    <row r="27" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
@@ -1017,31 +1162,37 @@
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="18">
-    <mergeCell ref="B16:K16"/>
+  <mergeCells count="22">
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:L5"/>
+    <mergeCell ref="M4:M5"/>
+    <mergeCell ref="B2:M2"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="J4:J5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
+    <mergeCell ref="B16:M16"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="C18:C19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:G18"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="F18:F19"/>
+    <mergeCell ref="G18:I18"/>
     <mergeCell ref="J18:J19"/>
     <mergeCell ref="K18:K19"/>
-    <mergeCell ref="I4:I5"/>
-    <mergeCell ref="J4:J5"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="B2:K2"/>
-    <mergeCell ref="E4:G4"/>
-    <mergeCell ref="H4:H5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="L18:L19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="D18:D19"/>
+    <mergeCell ref="E18:E19"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K4" r:id="rId1"/>
-    <hyperlink ref="K18" r:id="rId2"/>
+    <hyperlink ref="M4" r:id="rId1"/>
+    <hyperlink ref="M18" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>

</xml_diff>

<commit_message>
wakes anotated and trained
</commit_message>
<xml_diff>
--- a/documentation/Training statistics.xlsx
+++ b/documentation/Training statistics.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="35">
   <si>
     <t>Training experiments - Chokepoint camera</t>
   </si>
@@ -123,6 +123,12 @@
   </si>
   <si>
     <t>Automatic</t>
+  </si>
+  <si>
+    <t>Roboflow (wakes annotated)</t>
+  </si>
+  <si>
+    <t>Manually trained(wakes annotated)</t>
   </si>
 </sst>
 </file>
@@ -252,13 +258,19 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -275,12 +287,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -563,7 +569,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:O27"/>
+  <dimension ref="B2:O28"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="11.08984375" customWidth="1"/>
@@ -574,61 +580,61 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
+      <c r="I2" s="8"/>
+      <c r="J2" s="8"/>
+      <c r="K2" s="8"/>
+      <c r="L2" s="8"/>
+      <c r="M2" s="8"/>
     </row>
     <row r="4" spans="2:15" ht="18" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F4" s="5" t="s">
+      <c r="F4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="9"/>
-      <c r="J4" s="10" t="s">
+      <c r="H4" s="10"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="K4" s="5" t="s">
+      <c r="K4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L4" s="5" t="s">
+      <c r="L4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M4" s="12" t="s">
+      <c r="M4" s="6" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="2:15" ht="29.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
       <c r="G5" s="2" t="s">
         <v>5</v>
       </c>
@@ -638,10 +644,10 @@
       <c r="I5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J5" s="11"/>
-      <c r="K5" s="6"/>
-      <c r="L5" s="6"/>
-      <c r="M5" s="13"/>
+      <c r="J5" s="13"/>
+      <c r="K5" s="5"/>
+      <c r="L5" s="5"/>
+      <c r="M5" s="7"/>
     </row>
     <row r="6" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="3">
@@ -918,137 +924,155 @@
         <v>0.442</v>
       </c>
     </row>
-    <row r="13" spans="2:15" ht="13" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+    <row r="13" spans="2:15" x14ac:dyDescent="0.35">
+      <c r="B13" s="3">
+        <v>46092</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>34</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
-      <c r="F13" s="1"/>
-      <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-      <c r="J13" s="1"/>
-      <c r="K13" s="1"/>
-      <c r="L13" s="1"/>
-      <c r="M13" s="1"/>
-    </row>
-    <row r="16" spans="2:15" x14ac:dyDescent="0.35">
-      <c r="B16" s="4" t="s">
+      <c r="F13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="1">
+        <v>236</v>
+      </c>
+      <c r="H13" s="1">
+        <v>114</v>
+      </c>
+      <c r="I13" s="1">
+        <v>49</v>
+      </c>
+      <c r="J13" s="1">
+        <v>871</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0.35099999999999998</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0.54</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="14" spans="2:15" ht="13" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="3">
+        <v>46092</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G14" s="1">
+        <v>236</v>
+      </c>
+      <c r="H14" s="1">
+        <v>114</v>
+      </c>
+      <c r="I14" s="1">
+        <v>49</v>
+      </c>
+      <c r="J14" s="1">
+        <v>871</v>
+      </c>
+      <c r="K14" s="1">
+        <v>0.56799999999999995</v>
+      </c>
+      <c r="L14" s="1">
+        <v>0.42799999999999999</v>
+      </c>
+      <c r="M14" s="1">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="17" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B17" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4"/>
-      <c r="K16" s="4"/>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-    </row>
-    <row r="18" spans="2:14" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="5" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+    </row>
+    <row r="19" spans="2:14" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B19" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C19" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="E19" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="5" t="s">
+      <c r="F19" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G18" s="7" t="s">
+      <c r="G19" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="8"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="10" t="s">
+      <c r="H19" s="10"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="K18" s="5" t="s">
+      <c r="K19" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L18" s="5" t="s">
+      <c r="L19" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="M18" s="12" t="s">
+      <c r="M19" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="2:14" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6"/>
-      <c r="G19" s="2" t="s">
+    <row r="20" spans="2:14" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="5"/>
+      <c r="C20" s="5"/>
+      <c r="D20" s="5"/>
+      <c r="E20" s="5"/>
+      <c r="F20" s="5"/>
+      <c r="G20" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="H19" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="I19" s="2" t="s">
+      <c r="I20" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="J19" s="11"/>
-      <c r="K19" s="6"/>
-      <c r="L19" s="6"/>
-      <c r="M19" s="13"/>
-    </row>
-    <row r="20" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B20" s="3">
-        <v>46071</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="E20" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F20" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="1">
-        <v>88</v>
-      </c>
-      <c r="H20" s="1">
-        <v>25</v>
-      </c>
-      <c r="I20" s="1">
-        <v>12</v>
-      </c>
-      <c r="J20" s="1">
-        <v>301</v>
-      </c>
-      <c r="K20" s="1">
-        <v>0.93200000000000005</v>
-      </c>
-      <c r="L20" s="1">
-        <v>0.72499999999999998</v>
-      </c>
-      <c r="M20" s="1">
-        <v>0.82599999999999996</v>
-      </c>
+      <c r="J20" s="13"/>
+      <c r="K20" s="5"/>
+      <c r="L20" s="5"/>
+      <c r="M20" s="7"/>
     </row>
     <row r="21" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B21" s="3">
-        <v>46072</v>
+        <v>46071</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>11</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>32</v>
@@ -1057,43 +1081,67 @@
         <v>13</v>
       </c>
       <c r="G21" s="1">
+        <v>88</v>
+      </c>
+      <c r="H21" s="1">
+        <v>25</v>
+      </c>
+      <c r="I21" s="1">
+        <v>12</v>
+      </c>
+      <c r="J21" s="1">
+        <v>301</v>
+      </c>
+      <c r="K21" s="1">
+        <v>0.93200000000000005</v>
+      </c>
+      <c r="L21" s="1">
+        <v>0.72499999999999998</v>
+      </c>
+      <c r="M21" s="1">
+        <v>0.82599999999999996</v>
+      </c>
+    </row>
+    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B22" s="3">
+        <v>46072</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="1">
         <v>189</v>
       </c>
-      <c r="H21" s="1">
+      <c r="H22" s="1">
         <v>72</v>
       </c>
-      <c r="I21" s="1">
+      <c r="I22" s="1">
         <v>31</v>
       </c>
-      <c r="J21" s="1">
+      <c r="J22" s="1">
         <v>704</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K22" s="1">
         <v>0.94099999999999995</v>
       </c>
-      <c r="L21" s="1">
+      <c r="L22" s="1">
         <v>0.79600000000000004</v>
       </c>
-      <c r="M21" s="1">
+      <c r="M22" s="1">
         <v>0.88700000000000001</v>
       </c>
-      <c r="N21" t="s">
+      <c r="N22" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="22" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B22" s="3"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
-      <c r="F22" s="1"/>
-      <c r="G22" s="1"/>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="1"/>
-      <c r="M22" s="1"/>
     </row>
     <row r="23" spans="2:14" x14ac:dyDescent="0.35">
       <c r="B23" s="3"/>
@@ -1124,7 +1172,7 @@
       <c r="M24" s="1"/>
     </row>
     <row r="25" spans="2:14" x14ac:dyDescent="0.35">
-      <c r="B25" s="1"/>
+      <c r="B25" s="3"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
@@ -1165,8 +1213,33 @@
       <c r="L27" s="1"/>
       <c r="M27" s="1"/>
     </row>
+    <row r="28" spans="2:14" x14ac:dyDescent="0.35">
+      <c r="B28" s="1"/>
+      <c r="C28" s="1"/>
+      <c r="D28" s="1"/>
+      <c r="E28" s="1"/>
+      <c r="F28" s="1"/>
+      <c r="G28" s="1"/>
+      <c r="H28" s="1"/>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+    </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="B17:M17"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="C19:C20"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="G19:I19"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="K19:K20"/>
+    <mergeCell ref="L19:L20"/>
+    <mergeCell ref="M19:M20"/>
+    <mergeCell ref="D19:D20"/>
+    <mergeCell ref="E19:E20"/>
     <mergeCell ref="K4:K5"/>
     <mergeCell ref="L4:L5"/>
     <mergeCell ref="M4:M5"/>
@@ -1178,21 +1251,10 @@
     <mergeCell ref="F4:F5"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
-    <mergeCell ref="B16:M16"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="C18:C19"/>
-    <mergeCell ref="F18:F19"/>
-    <mergeCell ref="G18:I18"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="L18:L19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="D18:D19"/>
-    <mergeCell ref="E18:E19"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="M4" r:id="rId1"/>
-    <hyperlink ref="M18" r:id="rId2"/>
+    <hyperlink ref="M19" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="1200" verticalDpi="1200" r:id="rId3"/>

</xml_diff>